<commit_message>
for & back feedback
</commit_message>
<xml_diff>
--- a/Data/output/reforms/output/reform_panel.xlsx
+++ b/Data/output/reforms/output/reform_panel.xlsx
@@ -29475,40 +29475,40 @@
         <v>2006</v>
       </c>
       <c r="D323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P323" t="n">
         <v>0</v>
@@ -29526,7 +29526,7 @@
         <v>0</v>
       </c>
       <c r="U323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V323" t="n">
         <v>0</v>
@@ -29544,10 +29544,10 @@
         <v>0</v>
       </c>
       <c r="AA323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB323" t="n">
-        <v>0</v>
+        <v>0.6035</v>
       </c>
     </row>
     <row r="324">
@@ -29565,13 +29565,13 @@
         <v>2007</v>
       </c>
       <c r="D324" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E324" t="n">
         <v>1</v>
       </c>
       <c r="F324" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G324" t="n">
         <v>1</v>
@@ -29589,13 +29589,13 @@
         <v>1</v>
       </c>
       <c r="L324" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M324" t="n">
         <v>1</v>
       </c>
       <c r="N324" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O324" t="n">
         <v>1</v>
@@ -29622,7 +29622,7 @@
         <v>0</v>
       </c>
       <c r="W324" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X324" t="n">
         <v>0</v>
@@ -29637,7 +29637,7 @@
         <v>0</v>
       </c>
       <c r="AB324" t="n">
-        <v>0.5716</v>
+        <v>0.552</v>
       </c>
     </row>
     <row r="325">
@@ -29655,16 +29655,16 @@
         <v>2008</v>
       </c>
       <c r="D325" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E325" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F325" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G325" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H325" t="n">
         <v>0</v>
@@ -29679,16 +29679,16 @@
         <v>0</v>
       </c>
       <c r="L325" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M325" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N325" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O325" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P325" t="n">
         <v>0</v>
@@ -29706,16 +29706,16 @@
         <v>0</v>
       </c>
       <c r="U325" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V325" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W325" t="n">
         <v>0</v>
       </c>
       <c r="X325" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y325" t="n">
         <v>0</v>
@@ -29724,10 +29724,10 @@
         <v>0</v>
       </c>
       <c r="AA325" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB325" t="n">
-        <v>0</v>
+        <v>0.427</v>
       </c>
     </row>
     <row r="326">
@@ -29745,37 +29745,37 @@
         <v>2009</v>
       </c>
       <c r="D326" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E326" t="n">
         <v>1</v>
       </c>
       <c r="F326" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G326" t="n">
         <v>1</v>
       </c>
       <c r="H326" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I326" t="n">
         <v>1</v>
       </c>
       <c r="J326" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K326" t="n">
         <v>1</v>
       </c>
       <c r="L326" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M326" t="n">
         <v>1</v>
       </c>
       <c r="N326" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O326" t="n">
         <v>1</v>
@@ -29796,7 +29796,7 @@
         <v>0</v>
       </c>
       <c r="U326" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V326" t="n">
         <v>1</v>
@@ -29814,10 +29814,10 @@
         <v>0</v>
       </c>
       <c r="AA326" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AB326" t="n">
-        <v>0.707</v>
+        <v>0.677</v>
       </c>
     </row>
     <row r="327">
@@ -29835,16 +29835,16 @@
         <v>2010</v>
       </c>
       <c r="D327" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E327" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F327" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G327" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H327" t="n">
         <v>0</v>
@@ -29859,16 +29859,16 @@
         <v>0</v>
       </c>
       <c r="L327" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M327" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N327" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O327" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P327" t="n">
         <v>0</v>
@@ -29889,7 +29889,7 @@
         <v>0</v>
       </c>
       <c r="V327" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W327" t="n">
         <v>0</v>
@@ -29907,7 +29907,7 @@
         <v>0</v>
       </c>
       <c r="AB327" t="n">
-        <v>0</v>
+        <v>0.3535</v>
       </c>
     </row>
     <row r="328">
@@ -30015,37 +30015,37 @@
         <v>2012</v>
       </c>
       <c r="D329" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E329" t="n">
         <v>1</v>
       </c>
       <c r="F329" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G329" t="n">
         <v>1</v>
       </c>
       <c r="H329" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I329" t="n">
         <v>1</v>
       </c>
       <c r="J329" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K329" t="n">
         <v>1</v>
       </c>
       <c r="L329" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M329" t="n">
         <v>1</v>
       </c>
       <c r="N329" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O329" t="n">
         <v>1</v>
@@ -30066,28 +30066,28 @@
         <v>0</v>
       </c>
       <c r="U329" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V329" t="n">
         <v>1</v>
       </c>
       <c r="W329" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X329" t="n">
         <v>0</v>
       </c>
       <c r="Y329" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z329" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA329" t="n">
         <v>1</v>
       </c>
-      <c r="Z329" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA329" t="n">
-        <v>0</v>
-      </c>
       <c r="AB329" t="n">
-        <v>0.6035</v>
+        <v>0.6052999999999999</v>
       </c>
     </row>
     <row r="330">
@@ -30105,37 +30105,37 @@
         <v>2013</v>
       </c>
       <c r="D330" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E330" t="n">
         <v>1</v>
       </c>
       <c r="F330" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G330" t="n">
         <v>1</v>
       </c>
       <c r="H330" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I330" t="n">
         <v>1</v>
       </c>
       <c r="J330" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K330" t="n">
         <v>1</v>
       </c>
       <c r="L330" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M330" t="n">
         <v>1</v>
       </c>
       <c r="N330" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O330" t="n">
         <v>1</v>
@@ -30162,7 +30162,7 @@
         <v>0</v>
       </c>
       <c r="W330" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X330" t="n">
         <v>0</v>
@@ -30174,10 +30174,10 @@
         <v>0</v>
       </c>
       <c r="AA330" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AB330" t="n">
-        <v>0.6237</v>
+        <v>0.6035</v>
       </c>
     </row>
     <row r="331">
@@ -42435,40 +42435,40 @@
         <v>1995</v>
       </c>
       <c r="D467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P467" t="n">
         <v>0</v>
@@ -42492,13 +42492,13 @@
         <v>0</v>
       </c>
       <c r="W467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X467" t="n">
         <v>0</v>
       </c>
       <c r="Y467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z467" t="n">
         <v>0</v>
@@ -42507,7 +42507,7 @@
         <v>0</v>
       </c>
       <c r="AB467" t="n">
-        <v>0</v>
+        <v>0.6035</v>
       </c>
     </row>
     <row r="468">
@@ -42885,40 +42885,40 @@
         <v>2000</v>
       </c>
       <c r="D472" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E472" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F472" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G472" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H472" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I472" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J472" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K472" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L472" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M472" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N472" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O472" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P472" t="n">
         <v>0</v>
@@ -42939,7 +42939,7 @@
         <v>0</v>
       </c>
       <c r="V472" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W472" t="n">
         <v>0</v>
@@ -42948,7 +42948,7 @@
         <v>0</v>
       </c>
       <c r="Y472" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z472" t="n">
         <v>0</v>
@@ -42957,7 +42957,7 @@
         <v>0</v>
       </c>
       <c r="AB472" t="n">
-        <v>0</v>
+        <v>0.5208</v>
       </c>
     </row>
     <row r="473">
@@ -43245,40 +43245,40 @@
         <v>2004</v>
       </c>
       <c r="D476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P476" t="n">
         <v>0</v>
@@ -43296,7 +43296,7 @@
         <v>0</v>
       </c>
       <c r="U476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V476" t="n">
         <v>0</v>
@@ -43305,7 +43305,7 @@
         <v>0</v>
       </c>
       <c r="X476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y476" t="n">
         <v>0</v>
@@ -43317,7 +43317,7 @@
         <v>0</v>
       </c>
       <c r="AB476" t="n">
-        <v>0</v>
+        <v>0.6035</v>
       </c>
     </row>
     <row r="477">
@@ -43335,40 +43335,40 @@
         <v>2005</v>
       </c>
       <c r="D477" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E477" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F477" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G477" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H477" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I477" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J477" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K477" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L477" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M477" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N477" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O477" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P477" t="n">
         <v>0</v>
@@ -43383,10 +43383,10 @@
         <v>0</v>
       </c>
       <c r="T477" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U477" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V477" t="n">
         <v>0</v>
@@ -43398,7 +43398,7 @@
         <v>0</v>
       </c>
       <c r="Y477" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z477" t="n">
         <v>0</v>
@@ -43407,7 +43407,7 @@
         <v>0</v>
       </c>
       <c r="AB477" t="n">
-        <v>0</v>
+        <v>0.677</v>
       </c>
     </row>
     <row r="478">
@@ -43473,7 +43473,7 @@
         <v>0</v>
       </c>
       <c r="T478" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U478" t="n">
         <v>0</v>
@@ -43515,40 +43515,40 @@
         <v>2007</v>
       </c>
       <c r="D479" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E479" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F479" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G479" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H479" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I479" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J479" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K479" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L479" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M479" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N479" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O479" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P479" t="n">
         <v>0</v>
@@ -43563,31 +43563,31 @@
         <v>0</v>
       </c>
       <c r="T479" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U479" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V479" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W479" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X479" t="n">
         <v>0</v>
       </c>
       <c r="Y479" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Z479" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA479" t="n">
         <v>0</v>
       </c>
       <c r="AB479" t="n">
-        <v>0</v>
+        <v>0.7615</v>
       </c>
     </row>
     <row r="480">
@@ -43605,40 +43605,40 @@
         <v>2008</v>
       </c>
       <c r="D480" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E480" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F480" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G480" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H480" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I480" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J480" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K480" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L480" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M480" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N480" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O480" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P480" t="n">
         <v>0</v>
@@ -43656,7 +43656,7 @@
         <v>0</v>
       </c>
       <c r="U480" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V480" t="n">
         <v>0</v>
@@ -43674,10 +43674,10 @@
         <v>0</v>
       </c>
       <c r="AA480" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB480" t="n">
-        <v>0</v>
+        <v>0.6035</v>
       </c>
     </row>
     <row r="481">
@@ -43785,40 +43785,40 @@
         <v>2010</v>
       </c>
       <c r="D482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P482" t="n">
         <v>0</v>
@@ -43836,7 +43836,7 @@
         <v>0</v>
       </c>
       <c r="U482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V482" t="n">
         <v>0</v>
@@ -43848,7 +43848,7 @@
         <v>0</v>
       </c>
       <c r="Y482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z482" t="n">
         <v>0</v>
@@ -43857,7 +43857,7 @@
         <v>0</v>
       </c>
       <c r="AB482" t="n">
-        <v>0</v>
+        <v>0.6035</v>
       </c>
     </row>
     <row r="483">
@@ -43875,16 +43875,16 @@
         <v>2011</v>
       </c>
       <c r="D483" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E483" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F483" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G483" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H483" t="n">
         <v>0</v>
@@ -43899,16 +43899,16 @@
         <v>0</v>
       </c>
       <c r="L483" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M483" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N483" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O483" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P483" t="n">
         <v>0</v>
@@ -43923,7 +43923,7 @@
         <v>0</v>
       </c>
       <c r="T483" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U483" t="n">
         <v>0</v>
@@ -43932,7 +43932,7 @@
         <v>0</v>
       </c>
       <c r="W483" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X483" t="n">
         <v>0</v>
@@ -43944,10 +43944,10 @@
         <v>0</v>
       </c>
       <c r="AA483" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB483" t="n">
-        <v>0</v>
+        <v>0.3535</v>
       </c>
     </row>
     <row r="484">
@@ -43965,40 +43965,40 @@
         <v>2012</v>
       </c>
       <c r="D484" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E484" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F484" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G484" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H484" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I484" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J484" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K484" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L484" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M484" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N484" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O484" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P484" t="n">
         <v>0</v>
@@ -44016,10 +44016,10 @@
         <v>0</v>
       </c>
       <c r="U484" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V484" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W484" t="n">
         <v>0</v>
@@ -44028,16 +44028,16 @@
         <v>0</v>
       </c>
       <c r="Y484" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z484" t="n">
         <v>0</v>
       </c>
       <c r="AA484" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB484" t="n">
-        <v>0</v>
+        <v>0.6237</v>
       </c>
     </row>
     <row r="485">
@@ -44103,7 +44103,7 @@
         <v>0</v>
       </c>
       <c r="T485" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U485" t="n">
         <v>0</v>
@@ -44235,40 +44235,40 @@
         <v>2015</v>
       </c>
       <c r="D487" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E487" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F487" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G487" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H487" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I487" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J487" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K487" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L487" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M487" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N487" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O487" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P487" t="n">
         <v>0</v>
@@ -44286,7 +44286,7 @@
         <v>0</v>
       </c>
       <c r="U487" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V487" t="n">
         <v>0</v>
@@ -44304,10 +44304,10 @@
         <v>0</v>
       </c>
       <c r="AA487" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB487" t="n">
-        <v>0</v>
+        <v>0.6035</v>
       </c>
     </row>
     <row r="488">
@@ -44415,16 +44415,16 @@
         <v>2017</v>
       </c>
       <c r="D489" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E489" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F489" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G489" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H489" t="n">
         <v>0</v>
@@ -44439,16 +44439,16 @@
         <v>0</v>
       </c>
       <c r="L489" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M489" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N489" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O489" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P489" t="n">
         <v>0</v>
@@ -44463,10 +44463,10 @@
         <v>0</v>
       </c>
       <c r="T489" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="U489" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V489" t="n">
         <v>0</v>
@@ -44484,10 +44484,10 @@
         <v>0</v>
       </c>
       <c r="AA489" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB489" t="n">
-        <v>0</v>
+        <v>0.3535</v>
       </c>
     </row>
     <row r="490">
@@ -44733,7 +44733,7 @@
         <v>0</v>
       </c>
       <c r="T492" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U492" t="n">
         <v>0</v>
@@ -44775,40 +44775,40 @@
         <v>2021</v>
       </c>
       <c r="D493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P493" t="n">
         <v>0</v>
@@ -44826,7 +44826,7 @@
         <v>0</v>
       </c>
       <c r="U493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V493" t="n">
         <v>0</v>
@@ -44838,7 +44838,7 @@
         <v>0</v>
       </c>
       <c r="Y493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z493" t="n">
         <v>0</v>
@@ -44847,7 +44847,7 @@
         <v>0</v>
       </c>
       <c r="AB493" t="n">
-        <v>0</v>
+        <v>0.6035</v>
       </c>
     </row>
     <row r="494">

</xml_diff>

<commit_message>
forwad and back in budget
</commit_message>
<xml_diff>
--- a/Data/output/reforms/output/reform_panel.xlsx
+++ b/Data/output/reforms/output/reform_panel.xlsx
@@ -30015,13 +30015,13 @@
         <v>2012</v>
       </c>
       <c r="D329" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E329" t="n">
         <v>1</v>
       </c>
       <c r="F329" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G329" t="n">
         <v>1</v>
@@ -30039,13 +30039,13 @@
         <v>1</v>
       </c>
       <c r="L329" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M329" t="n">
         <v>1</v>
       </c>
       <c r="N329" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O329" t="n">
         <v>1</v>
@@ -30066,13 +30066,13 @@
         <v>0</v>
       </c>
       <c r="U329" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V329" t="n">
         <v>1</v>
       </c>
       <c r="W329" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X329" t="n">
         <v>0</v>
@@ -30084,10 +30084,10 @@
         <v>0</v>
       </c>
       <c r="AA329" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB329" t="n">
-        <v>0.6052999999999999</v>
+        <v>0.6237</v>
       </c>
     </row>
     <row r="330">
@@ -30195,40 +30195,40 @@
         <v>2014</v>
       </c>
       <c r="D331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P331" t="n">
         <v>0</v>
@@ -30246,7 +30246,7 @@
         <v>0</v>
       </c>
       <c r="U331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V331" t="n">
         <v>0</v>
@@ -30255,7 +30255,7 @@
         <v>0</v>
       </c>
       <c r="X331" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y331" t="n">
         <v>0</v>
@@ -30267,7 +30267,7 @@
         <v>0</v>
       </c>
       <c r="AB331" t="n">
-        <v>0.6035</v>
+        <v>0</v>
       </c>
     </row>
     <row r="332">

</xml_diff>

<commit_message>
reforms 10 countries done
</commit_message>
<xml_diff>
--- a/Data/output/reforms/output/reform_panel.xlsx
+++ b/Data/output/reforms/output/reform_panel.xlsx
@@ -42435,13 +42435,13 @@
         <v>1995</v>
       </c>
       <c r="D467" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E467" t="n">
         <v>1</v>
       </c>
       <c r="F467" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G467" t="n">
         <v>1</v>
@@ -42459,13 +42459,13 @@
         <v>1</v>
       </c>
       <c r="L467" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M467" t="n">
         <v>1</v>
       </c>
       <c r="N467" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O467" t="n">
         <v>1</v>
@@ -42492,7 +42492,7 @@
         <v>0</v>
       </c>
       <c r="W467" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X467" t="n">
         <v>0</v>
@@ -42504,10 +42504,10 @@
         <v>0</v>
       </c>
       <c r="AA467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB467" t="n">
-        <v>0.6035</v>
+        <v>0.552</v>
       </c>
     </row>
     <row r="468">
@@ -42525,40 +42525,40 @@
         <v>1996</v>
       </c>
       <c r="D468" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F468" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L468" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N468" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P468" t="n">
         <v>0</v>
@@ -42573,31 +42573,31 @@
         <v>0</v>
       </c>
       <c r="T468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U468" t="n">
         <v>0</v>
       </c>
       <c r="V468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W468" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X468" t="n">
         <v>0</v>
       </c>
       <c r="Y468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB468" t="n">
-        <v>0</v>
+        <v>0.5404</v>
       </c>
     </row>
     <row r="469">
@@ -42705,40 +42705,40 @@
         <v>1998</v>
       </c>
       <c r="D470" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E470" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F470" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G470" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H470" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I470" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J470" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K470" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L470" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M470" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N470" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O470" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P470" t="n">
         <v>0</v>
@@ -42753,31 +42753,31 @@
         <v>0</v>
       </c>
       <c r="T470" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U470" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V470" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W470" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X470" t="n">
         <v>0</v>
       </c>
       <c r="Y470" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z470" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA470" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB470" t="n">
-        <v>0</v>
+        <v>0.7615</v>
       </c>
     </row>
     <row r="471">
@@ -42795,40 +42795,40 @@
         <v>1999</v>
       </c>
       <c r="D471" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E471" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F471" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G471" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H471" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I471" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J471" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K471" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L471" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M471" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N471" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O471" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P471" t="n">
         <v>0</v>
@@ -42846,10 +42846,10 @@
         <v>0</v>
       </c>
       <c r="U471" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V471" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W471" t="n">
         <v>0</v>
@@ -42858,7 +42858,7 @@
         <v>0</v>
       </c>
       <c r="Y471" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z471" t="n">
         <v>0</v>
@@ -42867,7 +42867,7 @@
         <v>0</v>
       </c>
       <c r="AB471" t="n">
-        <v>0</v>
+        <v>0.552</v>
       </c>
     </row>
     <row r="472">
@@ -42885,37 +42885,37 @@
         <v>2000</v>
       </c>
       <c r="D472" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E472" t="n">
         <v>1</v>
       </c>
       <c r="F472" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G472" t="n">
         <v>1</v>
       </c>
       <c r="H472" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I472" t="n">
         <v>1</v>
       </c>
       <c r="J472" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K472" t="n">
         <v>1</v>
       </c>
       <c r="L472" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M472" t="n">
         <v>1</v>
       </c>
       <c r="N472" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O472" t="n">
         <v>1</v>
@@ -42933,31 +42933,31 @@
         <v>0</v>
       </c>
       <c r="T472" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U472" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V472" t="n">
         <v>2</v>
       </c>
       <c r="W472" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X472" t="n">
         <v>0</v>
       </c>
       <c r="Y472" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z472" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA472" t="n">
         <v>2</v>
       </c>
-      <c r="Z472" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA472" t="n">
-        <v>0</v>
-      </c>
       <c r="AB472" t="n">
-        <v>0.5208</v>
+        <v>0.7133</v>
       </c>
     </row>
     <row r="473">
@@ -43065,16 +43065,16 @@
         <v>2002</v>
       </c>
       <c r="D474" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E474" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F474" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G474" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H474" t="n">
         <v>0</v>
@@ -43089,16 +43089,16 @@
         <v>0</v>
       </c>
       <c r="L474" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M474" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N474" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O474" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P474" t="n">
         <v>0</v>
@@ -43113,13 +43113,13 @@
         <v>0</v>
       </c>
       <c r="T474" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U474" t="n">
         <v>0</v>
       </c>
       <c r="V474" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W474" t="n">
         <v>0</v>
@@ -43134,10 +43134,10 @@
         <v>0</v>
       </c>
       <c r="AA474" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB474" t="n">
-        <v>0</v>
+        <v>0.3535</v>
       </c>
     </row>
     <row r="475">
@@ -43155,40 +43155,40 @@
         <v>2003</v>
       </c>
       <c r="D475" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E475" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F475" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G475" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H475" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I475" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J475" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K475" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L475" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M475" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N475" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O475" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P475" t="n">
         <v>0</v>
@@ -43206,28 +43206,28 @@
         <v>0</v>
       </c>
       <c r="U475" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V475" t="n">
         <v>0</v>
       </c>
       <c r="W475" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X475" t="n">
         <v>0</v>
       </c>
       <c r="Y475" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z475" t="n">
         <v>0</v>
       </c>
       <c r="AA475" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB475" t="n">
-        <v>0</v>
+        <v>0.677</v>
       </c>
     </row>
     <row r="476">
@@ -43293,7 +43293,7 @@
         <v>0</v>
       </c>
       <c r="T476" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U476" t="n">
         <v>1</v>
@@ -43305,10 +43305,10 @@
         <v>0</v>
       </c>
       <c r="X476" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y476" t="n">
         <v>1</v>
-      </c>
-      <c r="Y476" t="n">
-        <v>0</v>
       </c>
       <c r="Z476" t="n">
         <v>0</v>
@@ -43473,7 +43473,7 @@
         <v>0</v>
       </c>
       <c r="T478" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U478" t="n">
         <v>0</v>
@@ -43515,37 +43515,37 @@
         <v>2007</v>
       </c>
       <c r="D479" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E479" t="n">
         <v>1</v>
       </c>
       <c r="F479" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G479" t="n">
         <v>1</v>
       </c>
       <c r="H479" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I479" t="n">
         <v>1</v>
       </c>
       <c r="J479" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K479" t="n">
         <v>1</v>
       </c>
       <c r="L479" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M479" t="n">
         <v>1</v>
       </c>
       <c r="N479" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O479" t="n">
         <v>1</v>
@@ -43569,7 +43569,7 @@
         <v>1</v>
       </c>
       <c r="V479" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W479" t="n">
         <v>1</v>
@@ -43578,7 +43578,7 @@
         <v>0</v>
       </c>
       <c r="Y479" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Z479" t="n">
         <v>1</v>
@@ -43587,7 +43587,7 @@
         <v>0</v>
       </c>
       <c r="AB479" t="n">
-        <v>0.7615</v>
+        <v>0.6549</v>
       </c>
     </row>
     <row r="480">
@@ -43605,40 +43605,40 @@
         <v>2008</v>
       </c>
       <c r="D480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P480" t="n">
         <v>0</v>
@@ -43656,7 +43656,7 @@
         <v>0</v>
       </c>
       <c r="U480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V480" t="n">
         <v>0</v>
@@ -43674,10 +43674,10 @@
         <v>0</v>
       </c>
       <c r="AA480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB480" t="n">
-        <v>0.6035</v>
+        <v>0</v>
       </c>
     </row>
     <row r="481">
@@ -43785,40 +43785,40 @@
         <v>2010</v>
       </c>
       <c r="D482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P482" t="n">
         <v>0</v>
@@ -43836,7 +43836,7 @@
         <v>0</v>
       </c>
       <c r="U482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V482" t="n">
         <v>0</v>
@@ -43848,7 +43848,7 @@
         <v>0</v>
       </c>
       <c r="Y482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z482" t="n">
         <v>0</v>
@@ -43857,7 +43857,7 @@
         <v>0</v>
       </c>
       <c r="AB482" t="n">
-        <v>0.6035</v>
+        <v>0</v>
       </c>
     </row>
     <row r="483">
@@ -43875,16 +43875,16 @@
         <v>2011</v>
       </c>
       <c r="D483" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E483" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F483" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G483" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H483" t="n">
         <v>0</v>
@@ -43899,16 +43899,16 @@
         <v>0</v>
       </c>
       <c r="L483" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M483" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N483" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O483" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P483" t="n">
         <v>0</v>
@@ -43932,7 +43932,7 @@
         <v>0</v>
       </c>
       <c r="W483" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X483" t="n">
         <v>0</v>
@@ -43944,10 +43944,10 @@
         <v>0</v>
       </c>
       <c r="AA483" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB483" t="n">
-        <v>0.3535</v>
+        <v>0</v>
       </c>
     </row>
     <row r="484">
@@ -44055,40 +44055,40 @@
         <v>2013</v>
       </c>
       <c r="D485" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E485" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F485" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G485" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H485" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I485" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J485" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K485" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L485" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M485" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N485" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O485" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P485" t="n">
         <v>0</v>
@@ -44112,7 +44112,7 @@
         <v>0</v>
       </c>
       <c r="W485" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X485" t="n">
         <v>0</v>
@@ -44127,7 +44127,7 @@
         <v>0</v>
       </c>
       <c r="AB485" t="n">
-        <v>0</v>
+        <v>0.6035</v>
       </c>
     </row>
     <row r="486">
@@ -44415,13 +44415,13 @@
         <v>2017</v>
       </c>
       <c r="D489" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E489" t="n">
         <v>1</v>
       </c>
       <c r="F489" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G489" t="n">
         <v>1</v>
@@ -44439,13 +44439,13 @@
         <v>0</v>
       </c>
       <c r="L489" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M489" t="n">
         <v>1</v>
       </c>
       <c r="N489" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O489" t="n">
         <v>1</v>
@@ -44472,7 +44472,7 @@
         <v>0</v>
       </c>
       <c r="W489" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X489" t="n">
         <v>0</v>
@@ -44484,10 +44484,10 @@
         <v>0</v>
       </c>
       <c r="AA489" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AB489" t="n">
-        <v>0.3535</v>
+        <v>0.427</v>
       </c>
     </row>
     <row r="490">
@@ -44505,16 +44505,16 @@
         <v>2018</v>
       </c>
       <c r="D490" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E490" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F490" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G490" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H490" t="n">
         <v>0</v>
@@ -44529,16 +44529,16 @@
         <v>0</v>
       </c>
       <c r="L490" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M490" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N490" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O490" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P490" t="n">
         <v>0</v>
@@ -44562,7 +44562,7 @@
         <v>0</v>
       </c>
       <c r="W490" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X490" t="n">
         <v>0</v>
@@ -44574,10 +44574,10 @@
         <v>0</v>
       </c>
       <c r="AA490" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB490" t="n">
-        <v>0</v>
+        <v>0.3535</v>
       </c>
     </row>
     <row r="491">
@@ -44685,40 +44685,40 @@
         <v>2020</v>
       </c>
       <c r="D492" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E492" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F492" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G492" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H492" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I492" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J492" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K492" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L492" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M492" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N492" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O492" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P492" t="n">
         <v>0</v>
@@ -44733,22 +44733,22 @@
         <v>0</v>
       </c>
       <c r="T492" t="n">
+        <v>8</v>
+      </c>
+      <c r="U492" t="n">
+        <v>4</v>
+      </c>
+      <c r="V492" t="n">
         <v>1</v>
       </c>
-      <c r="U492" t="n">
-        <v>0</v>
-      </c>
-      <c r="V492" t="n">
-        <v>0</v>
-      </c>
       <c r="W492" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X492" t="n">
         <v>0</v>
       </c>
       <c r="Y492" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z492" t="n">
         <v>0</v>
@@ -44757,7 +44757,7 @@
         <v>0</v>
       </c>
       <c r="AB492" t="n">
-        <v>0</v>
+        <v>0.7029</v>
       </c>
     </row>
     <row r="493">
@@ -44775,37 +44775,37 @@
         <v>2021</v>
       </c>
       <c r="D493" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E493" t="n">
         <v>1</v>
       </c>
       <c r="F493" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G493" t="n">
         <v>1</v>
       </c>
       <c r="H493" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I493" t="n">
         <v>1</v>
       </c>
       <c r="J493" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K493" t="n">
         <v>1</v>
       </c>
       <c r="L493" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M493" t="n">
         <v>1</v>
       </c>
       <c r="N493" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O493" t="n">
         <v>1</v>
@@ -44823,13 +44823,13 @@
         <v>0</v>
       </c>
       <c r="T493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U493" t="n">
         <v>1</v>
       </c>
       <c r="V493" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W493" t="n">
         <v>0</v>
@@ -44838,7 +44838,7 @@
         <v>0</v>
       </c>
       <c r="Y493" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z493" t="n">
         <v>0</v>
@@ -44847,7 +44847,7 @@
         <v>0</v>
       </c>
       <c r="AB493" t="n">
-        <v>0.6035</v>
+        <v>0.677</v>
       </c>
     </row>
     <row r="494">
@@ -44865,40 +44865,40 @@
         <v>2022</v>
       </c>
       <c r="D494" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E494" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F494" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G494" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H494" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I494" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J494" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K494" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L494" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M494" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N494" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O494" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P494" t="n">
         <v>0</v>
@@ -44913,31 +44913,31 @@
         <v>0</v>
       </c>
       <c r="T494" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="U494" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V494" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W494" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X494" t="n">
         <v>0</v>
       </c>
       <c r="Y494" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z494" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA494" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB494" t="n">
-        <v>0</v>
+        <v>0.6549</v>
       </c>
     </row>
     <row r="495">
@@ -44955,40 +44955,40 @@
         <v>2023</v>
       </c>
       <c r="D495" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E495" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F495" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G495" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H495" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I495" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J495" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K495" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L495" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M495" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N495" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O495" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P495" t="n">
         <v>0</v>
@@ -45003,13 +45003,13 @@
         <v>0</v>
       </c>
       <c r="T495" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U495" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V495" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W495" t="n">
         <v>0</v>
@@ -45018,16 +45018,16 @@
         <v>0</v>
       </c>
       <c r="Y495" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z495" t="n">
         <v>0</v>
       </c>
       <c r="AA495" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AB495" t="n">
-        <v>0</v>
+        <v>0.6237</v>
       </c>
     </row>
     <row r="496">
@@ -45045,40 +45045,40 @@
         <v>2024</v>
       </c>
       <c r="D496" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E496" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F496" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G496" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H496" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I496" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J496" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K496" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L496" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M496" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N496" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O496" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P496" t="n">
         <v>0</v>
@@ -45093,7 +45093,7 @@
         <v>0</v>
       </c>
       <c r="T496" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U496" t="n">
         <v>0</v>
@@ -45102,7 +45102,7 @@
         <v>0</v>
       </c>
       <c r="W496" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X496" t="n">
         <v>0</v>
@@ -45114,10 +45114,10 @@
         <v>0</v>
       </c>
       <c r="AA496" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB496" t="n">
-        <v>0</v>
+        <v>0.6035</v>
       </c>
     </row>
     <row r="497">
@@ -45183,7 +45183,7 @@
         <v>0</v>
       </c>
       <c r="T497" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U497" t="n">
         <v>0</v>

</xml_diff>